<commit_message>
function  autosum and max
</commit_message>
<xml_diff>
--- a/Machine Learning and Big Data Engineer/Fundamentals of Data Analytics/Advanced Excel Techniques/Excel 2019 Advanced Functions/Practice data_1.xlsx
+++ b/Machine Learning and Big Data Engineer/Fundamentals of Data Analytics/Advanced Excel Techniques/Excel 2019 Advanced Functions/Practice data_1.xlsx
@@ -1,29 +1,44 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Excel Practice sheets\excel\Advanced_Excel_Trainer_Guide\Day-1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\suyas\Downloads\CODING(1)\L&amp;T EduTech\Machine Learning and Big Data Engineer\Fundamentals of Data Analytics\Advanced Excel Techniques\Excel 2019 Advanced Functions\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{180FF6DD-3317-48E7-93A5-28CD24785BDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="75" windowWidth="12240" windowHeight="7995"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet3" sheetId="3" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="5" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet3!$A$1:$E$100</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="134">
   <si>
     <t>Hardcopy</t>
   </si>
@@ -407,16 +422,40 @@
   </si>
   <si>
     <t>PRISM DIGITECH</t>
+  </si>
+  <si>
+    <t>Jan</t>
+  </si>
+  <si>
+    <t>Feb</t>
+  </si>
+  <si>
+    <t>Mar</t>
+  </si>
+  <si>
+    <t>Apr</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>Jun</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -462,9 +501,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -502,9 +541,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -539,7 +578,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -574,7 +613,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -747,19 +786,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:E100"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="51" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -776,7 +815,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -793,7 +832,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -810,7 +849,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -827,7 +866,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -844,7 +883,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -861,7 +900,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -878,7 +917,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -895,7 +934,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -912,7 +951,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -929,7 +968,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -946,7 +985,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -963,7 +1002,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -980,7 +1019,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -997,7 +1036,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -1014,7 +1053,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>11</v>
       </c>
@@ -1031,7 +1070,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>11</v>
       </c>
@@ -1048,7 +1087,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>11</v>
       </c>
@@ -1065,7 +1104,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>11</v>
       </c>
@@ -1082,7 +1121,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>11</v>
       </c>
@@ -1099,7 +1138,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>11</v>
       </c>
@@ -1116,7 +1155,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>11</v>
       </c>
@@ -1133,7 +1172,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>11</v>
       </c>
@@ -1150,7 +1189,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>11</v>
       </c>
@@ -1167,7 +1206,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>11</v>
       </c>
@@ -1184,7 +1223,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>11</v>
       </c>
@@ -1201,7 +1240,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>11</v>
       </c>
@@ -1218,7 +1257,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>11</v>
       </c>
@@ -1235,7 +1274,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>11</v>
       </c>
@@ -1252,7 +1291,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>11</v>
       </c>
@@ -1269,7 +1308,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>11</v>
       </c>
@@ -1286,7 +1325,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>11</v>
       </c>
@@ -1303,7 +1342,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>11</v>
       </c>
@@ -1320,7 +1359,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>11</v>
       </c>
@@ -1337,7 +1376,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>11</v>
       </c>
@@ -1354,7 +1393,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>5</v>
       </c>
@@ -1371,7 +1410,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>11</v>
       </c>
@@ -1388,7 +1427,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>11</v>
       </c>
@@ -1405,7 +1444,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>5</v>
       </c>
@@ -1422,7 +1461,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>11</v>
       </c>
@@ -1439,7 +1478,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>11</v>
       </c>
@@ -1456,7 +1495,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>11</v>
       </c>
@@ -1473,7 +1512,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>11</v>
       </c>
@@ -1490,7 +1529,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>11</v>
       </c>
@@ -1507,7 +1546,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>11</v>
       </c>
@@ -1524,7 +1563,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>11</v>
       </c>
@@ -1541,7 +1580,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>5</v>
       </c>
@@ -1558,7 +1597,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>11</v>
       </c>
@@ -1575,7 +1614,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>11</v>
       </c>
@@ -1592,7 +1631,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>11</v>
       </c>
@@ -1609,7 +1648,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>5</v>
       </c>
@@ -1626,7 +1665,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>11</v>
       </c>
@@ -1643,7 +1682,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>11</v>
       </c>
@@ -1660,7 +1699,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>5</v>
       </c>
@@ -1677,7 +1716,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>11</v>
       </c>
@@ -1694,7 +1733,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>11</v>
       </c>
@@ -1711,7 +1750,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>5</v>
       </c>
@@ -1728,7 +1767,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>11</v>
       </c>
@@ -1745,7 +1784,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>11</v>
       </c>
@@ -1762,7 +1801,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>11</v>
       </c>
@@ -1779,7 +1818,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>11</v>
       </c>
@@ -1796,7 +1835,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>11</v>
       </c>
@@ -1813,7 +1852,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>11</v>
       </c>
@@ -1830,7 +1869,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>11</v>
       </c>
@@ -1847,7 +1886,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>11</v>
       </c>
@@ -1864,7 +1903,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>11</v>
       </c>
@@ -1881,7 +1920,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>11</v>
       </c>
@@ -1898,7 +1937,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>11</v>
       </c>
@@ -1915,7 +1954,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>11</v>
       </c>
@@ -1932,7 +1971,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>11</v>
       </c>
@@ -1949,7 +1988,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>11</v>
       </c>
@@ -1966,7 +2005,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>11</v>
       </c>
@@ -1983,7 +2022,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>11</v>
       </c>
@@ -2000,7 +2039,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>5</v>
       </c>
@@ -2017,7 +2056,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>11</v>
       </c>
@@ -2034,7 +2073,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>11</v>
       </c>
@@ -2051,7 +2090,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>11</v>
       </c>
@@ -2068,7 +2107,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>11</v>
       </c>
@@ -2085,7 +2124,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>11</v>
       </c>
@@ -2102,7 +2141,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>11</v>
       </c>
@@ -2119,7 +2158,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>11</v>
       </c>
@@ -2136,7 +2175,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>11</v>
       </c>
@@ -2153,7 +2192,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>11</v>
       </c>
@@ -2170,7 +2209,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>11</v>
       </c>
@@ -2187,7 +2226,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>11</v>
       </c>
@@ -2204,7 +2243,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>11</v>
       </c>
@@ -2221,7 +2260,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>11</v>
       </c>
@@ -2238,7 +2277,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>11</v>
       </c>
@@ -2255,7 +2294,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>11</v>
       </c>
@@ -2272,7 +2311,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>11</v>
       </c>
@@ -2289,7 +2328,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>11</v>
       </c>
@@ -2306,7 +2345,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>11</v>
       </c>
@@ -2323,7 +2362,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>5</v>
       </c>
@@ -2340,7 +2379,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>11</v>
       </c>
@@ -2357,7 +2396,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>11</v>
       </c>
@@ -2374,7 +2413,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>11</v>
       </c>
@@ -2391,7 +2430,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>5</v>
       </c>
@@ -2408,7 +2447,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>11</v>
       </c>
@@ -2425,7 +2464,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>11</v>
       </c>
@@ -2442,7 +2481,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>11</v>
       </c>
@@ -2465,11 +2504,185 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1">
+        <v>1</v>
+      </c>
+      <c r="E1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="G2" t="s">
+        <v>128</v>
+      </c>
+      <c r="H2" t="s">
+        <v>129</v>
+      </c>
+      <c r="I2" t="s">
+        <v>130</v>
+      </c>
+      <c r="J2" t="s">
+        <v>131</v>
+      </c>
+      <c r="K2" t="s">
+        <v>132</v>
+      </c>
+      <c r="L2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>3</v>
+      </c>
+      <c r="E3">
+        <v>6</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>3</v>
+      </c>
+      <c r="J3">
+        <v>4</v>
+      </c>
+      <c r="K3">
+        <v>5</v>
+      </c>
+      <c r="L3">
+        <f>SUM(G3:K3)</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>4</v>
+      </c>
+      <c r="E4">
+        <v>8</v>
+      </c>
+      <c r="G4">
+        <v>2</v>
+      </c>
+      <c r="H4">
+        <v>4</v>
+      </c>
+      <c r="I4">
+        <v>6</v>
+      </c>
+      <c r="J4">
+        <v>8</v>
+      </c>
+      <c r="K4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <f>SUM(A1:A4,Sheet1!B2:D2,PI())</f>
+        <v>19.141592653589793</v>
+      </c>
+      <c r="E5">
+        <v>10</v>
+      </c>
+      <c r="G5">
+        <v>3</v>
+      </c>
+      <c r="H5">
+        <v>6</v>
+      </c>
+      <c r="I5">
+        <v>9</v>
+      </c>
+      <c r="J5">
+        <v>12</v>
+      </c>
+      <c r="K5">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C6">
+        <f>PI()</f>
+        <v>3.1415926535897931</v>
+      </c>
+      <c r="E6">
+        <v>12</v>
+      </c>
+      <c r="G6">
+        <v>4</v>
+      </c>
+      <c r="H6">
+        <v>8</v>
+      </c>
+      <c r="I6">
+        <v>12</v>
+      </c>
+      <c r="J6">
+        <v>16</v>
+      </c>
+      <c r="K6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="E7">
+        <v>14</v>
+      </c>
+      <c r="G7">
+        <f>MAX(G3:G6)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="E8">
+        <f>_xlfn.STDEV.S(E1:E7)</f>
+        <v>4.3204937989385739</v>
+      </c>
+      <c r="G8">
+        <f>COUNT(G3:G6)</f>
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F5DB804-8CE0-4E4F-B457-10BE9CC8D0FC}">
+  <dimension ref="B2:D2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>